<commit_message>
Properties / Swap fix
</commit_message>
<xml_diff>
--- a/docs/todo/ThirdOrder/Details.xlsx
+++ b/docs/todo/ThirdOrder/Details.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Storage\Dev\SpiroAnim\docs\todo\ThirdOrder\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DD013FC9-8A5E-4920-972D-0DFAAFAC8DAC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5F0971EC-E524-44F2-8F05-563624C7A2B3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28695" yWindow="0" windowWidth="29010" windowHeight="17385" xr2:uid="{8B601632-AE46-456F-A341-F0547A8975C7}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="99" uniqueCount="18">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="126" uniqueCount="21">
   <si>
     <t>1:1</t>
   </si>
@@ -93,6 +93,15 @@
   </si>
   <si>
     <t>1-1</t>
+  </si>
+  <si>
+    <t>Hand: Anti / Prop: Spin / v1</t>
+  </si>
+  <si>
+    <t>Hand: Anti / Prop: Spin / v2</t>
+  </si>
+  <si>
+    <t>Hand: Anti / Prop: Spin / v3</t>
   </si>
 </sst>
 </file>
@@ -516,7 +525,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1641CA09-2AE3-48CA-8CBE-A6B68A53DAEE}">
-  <dimension ref="A5:Z9"/>
+  <dimension ref="A5:Z15"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="8" width="9.140625" style="1"/>
@@ -852,8 +861,197 @@
         <v>13</v>
       </c>
     </row>
+    <row r="11" spans="1:26" x14ac:dyDescent="0.25">
+      <c r="A11" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="B11" s="2"/>
+      <c r="C11" s="2"/>
+      <c r="D11" s="2"/>
+      <c r="E11" s="2"/>
+      <c r="F11" s="2"/>
+      <c r="G11" s="2"/>
+      <c r="H11" s="2"/>
+      <c r="J11" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="K11" s="2"/>
+      <c r="L11" s="2"/>
+      <c r="M11" s="2"/>
+      <c r="N11" s="2"/>
+      <c r="O11" s="2"/>
+      <c r="P11" s="2"/>
+      <c r="Q11" s="2"/>
+      <c r="S11" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="T11" s="2"/>
+      <c r="U11" s="2"/>
+      <c r="V11" s="2"/>
+      <c r="W11" s="2"/>
+      <c r="X11" s="2"/>
+      <c r="Y11" s="2"/>
+      <c r="Z11" s="2"/>
+    </row>
+    <row r="12" spans="1:26" x14ac:dyDescent="0.25">
+      <c r="A12" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B12" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="C12" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="D12" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E12" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F12" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="G12" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="H12" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="I12" s="1"/>
+      <c r="J12" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="K12" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="L12" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="M12" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="N12" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="O12" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="P12" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="Q12" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="R12" s="1"/>
+      <c r="S12" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="T12" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="U12" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="V12" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="W12" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="X12" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="Y12" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="Z12" s="1" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="13" spans="1:26" x14ac:dyDescent="0.25">
+      <c r="A13" s="3"/>
+      <c r="B13" s="3"/>
+      <c r="C13" s="3"/>
+      <c r="D13" s="3"/>
+      <c r="E13" s="3"/>
+      <c r="F13" s="3"/>
+      <c r="G13" s="3"/>
+      <c r="H13" s="3"/>
+      <c r="J13" s="3"/>
+      <c r="K13" s="3"/>
+      <c r="L13" s="3"/>
+      <c r="M13" s="3"/>
+      <c r="N13" s="3"/>
+      <c r="O13" s="3"/>
+      <c r="P13" s="3"/>
+      <c r="Q13" s="3"/>
+      <c r="S13" s="3"/>
+      <c r="T13" s="3"/>
+      <c r="U13" s="3"/>
+      <c r="V13" s="3"/>
+      <c r="W13" s="3"/>
+      <c r="X13" s="3"/>
+      <c r="Y13" s="3"/>
+      <c r="Z13" s="3"/>
+    </row>
+    <row r="14" spans="1:26" x14ac:dyDescent="0.25">
+      <c r="A14" s="5"/>
+      <c r="B14" s="5"/>
+      <c r="C14" s="5"/>
+      <c r="D14" s="5"/>
+      <c r="E14" s="5"/>
+      <c r="F14" s="5"/>
+      <c r="G14" s="5"/>
+      <c r="H14" s="5"/>
+      <c r="J14" s="5"/>
+      <c r="K14" s="5"/>
+      <c r="L14" s="5"/>
+      <c r="M14" s="5"/>
+      <c r="N14" s="5"/>
+      <c r="O14" s="5"/>
+      <c r="P14" s="5"/>
+      <c r="Q14" s="5"/>
+      <c r="S14" s="5"/>
+      <c r="T14" s="5"/>
+      <c r="U14" s="5"/>
+      <c r="V14" s="5"/>
+      <c r="W14" s="5"/>
+      <c r="X14" s="5"/>
+      <c r="Y14" s="5"/>
+      <c r="Z14" s="5"/>
+    </row>
+    <row r="15" spans="1:26" x14ac:dyDescent="0.25">
+      <c r="A15" s="4"/>
+      <c r="B15" s="4"/>
+      <c r="C15" s="4"/>
+      <c r="D15" s="4"/>
+      <c r="E15" s="4"/>
+      <c r="F15" s="4"/>
+      <c r="G15" s="4"/>
+      <c r="H15" s="4"/>
+      <c r="J15" s="4"/>
+      <c r="K15" s="4"/>
+      <c r="L15" s="4"/>
+      <c r="M15" s="4"/>
+      <c r="N15" s="4"/>
+      <c r="O15" s="4"/>
+      <c r="P15" s="4"/>
+      <c r="Q15" s="4"/>
+      <c r="S15" s="4"/>
+      <c r="T15" s="4"/>
+      <c r="U15" s="4"/>
+      <c r="V15" s="4"/>
+      <c r="W15" s="4"/>
+      <c r="X15" s="4"/>
+      <c r="Y15" s="4"/>
+      <c r="Z15" s="4"/>
+    </row>
   </sheetData>
-  <mergeCells count="3">
+  <mergeCells count="6">
+    <mergeCell ref="A11:H11"/>
+    <mergeCell ref="J11:Q11"/>
+    <mergeCell ref="S11:Z11"/>
     <mergeCell ref="S5:Z5"/>
     <mergeCell ref="J5:Q5"/>
     <mergeCell ref="A5:H5"/>

</xml_diff>